<commit_message>
11:18 am Thursday, 16 July 2026 (IST)
</commit_message>
<xml_diff>
--- a/All-Coding-Status-Friday, 10 July 2026.xlsx
+++ b/All-Coding-Status-Friday, 10 July 2026.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\akum1255\Desktop\Current Task Progress\Leaning Status\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6531A274-52FF-4F7D-9768-5B1BAE04E2B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51B69A79-7ABF-4F0E-9FD7-CAD6632B0D92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="791" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Java ☑" sheetId="1" r:id="rId1"/>
     <sheet name="Angular ☑" sheetId="2" r:id="rId2"/>
     <sheet name="SQL ☑" sheetId="3" r:id="rId3"/>
-    <sheet name="Project(Docker+Jenkins)" sheetId="4" r:id="rId4"/>
+    <sheet name="Project(Docker+Jenkins) ☑" sheetId="4" r:id="rId4"/>
     <sheet name="Spring -RameshF" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="141">
   <si>
     <t xml:space="preserve">Topic </t>
   </si>
@@ -558,6 +558,30 @@
   </si>
   <si>
     <t>Testing All</t>
+  </si>
+  <si>
+    <t>✅Section 1:Introduction</t>
+  </si>
+  <si>
+    <t>✅Section 2:Setting up Development Environment</t>
+  </si>
+  <si>
+    <t>✅Section 3:Setting up Development Environment</t>
+  </si>
+  <si>
+    <t>✅Section 4:REST API Fundamentals-Design REST APIs</t>
+  </si>
+  <si>
+    <t>✅Section 5:REST API Fundamentals-Best Practices</t>
+  </si>
+  <si>
+    <t>✅Section 6:REST API Fundamentals-Important Difference[Interview Question and Answer]</t>
+  </si>
+  <si>
+    <t>✅Section 7:REST API Role Plays</t>
+  </si>
+  <si>
+    <t>✅Section 8:Spring Boot REST API Development Basics</t>
   </si>
 </sst>
 </file>
@@ -605,7 +629,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -651,12 +675,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -727,7 +745,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -828,27 +846,6 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="18" fontId="0" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -857,6 +854,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1555,39 +1561,39 @@
       <c r="A2" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="34" t="s">
+      <c r="B2" s="37" t="s">
         <v>104</v>
       </c>
-      <c r="C2" s="35" t="s">
+      <c r="C2" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="35" t="s">
+      <c r="D2" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="36" t="s">
+      <c r="E2" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="37">
+      <c r="F2" s="32">
         <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="25" t="s">
         <v>11</v>
       </c>
       <c r="B3" s="38" t="s">
         <v>105</v>
       </c>
-      <c r="C3" s="35" t="s">
+      <c r="C3" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="35" t="s">
+      <c r="D3" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="35" t="s">
+      <c r="E3" s="30" t="s">
         <v>84</v>
       </c>
-      <c r="F3" s="37">
+      <c r="F3" s="32">
         <v>12</v>
       </c>
     </row>
@@ -1595,17 +1601,17 @@
       <c r="A4" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="40" t="s">
+      <c r="B4" s="39" t="s">
         <v>106</v>
       </c>
-      <c r="C4" s="35" t="s">
+      <c r="C4" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="35" t="s">
+      <c r="D4" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="35"/>
-      <c r="F4" s="37">
+      <c r="E4" s="30"/>
+      <c r="F4" s="32">
         <v>8</v>
       </c>
     </row>
@@ -1616,14 +1622,14 @@
       <c r="B5" s="38" t="s">
         <v>107</v>
       </c>
-      <c r="C5" s="35" t="s">
+      <c r="C5" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="35" t="s">
+      <c r="D5" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="E5" s="35"/>
-      <c r="F5" s="37">
+      <c r="E5" s="30"/>
+      <c r="F5" s="32">
         <v>8</v>
       </c>
     </row>
@@ -1634,14 +1640,14 @@
       <c r="B6" s="38" t="s">
         <v>108</v>
       </c>
-      <c r="C6" s="35" t="s">
+      <c r="C6" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="35" t="s">
+      <c r="D6" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="E6" s="35"/>
-      <c r="F6" s="37">
+      <c r="E6" s="30"/>
+      <c r="F6" s="32">
         <v>9</v>
       </c>
     </row>
@@ -1649,17 +1655,17 @@
       <c r="A7" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="40" t="s">
+      <c r="B7" s="39" t="s">
         <v>106</v>
       </c>
-      <c r="C7" s="35" t="s">
+      <c r="C7" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="35" t="s">
+      <c r="D7" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="35"/>
-      <c r="F7" s="37">
+      <c r="E7" s="30"/>
+      <c r="F7" s="32">
         <v>4</v>
       </c>
     </row>
@@ -1667,17 +1673,17 @@
       <c r="A8" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="B8" s="40" t="s">
+      <c r="B8" s="39" t="s">
         <v>106</v>
       </c>
-      <c r="C8" s="35" t="s">
+      <c r="C8" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="35" t="s">
+      <c r="D8" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="35"/>
-      <c r="F8" s="37">
+      <c r="E8" s="30"/>
+      <c r="F8" s="32">
         <v>4</v>
       </c>
     </row>
@@ -1685,17 +1691,17 @@
       <c r="A9" s="25" t="s">
         <v>34</v>
       </c>
-      <c r="B9" s="40" t="s">
+      <c r="B9" s="39" t="s">
         <v>106</v>
       </c>
-      <c r="C9" s="35" t="s">
+      <c r="C9" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="D9" s="35" t="s">
+      <c r="D9" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="E9" s="35"/>
-      <c r="F9" s="37">
+      <c r="E9" s="30"/>
+      <c r="F9" s="32">
         <v>2</v>
       </c>
     </row>
@@ -1703,17 +1709,17 @@
       <c r="A10" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="B10" s="40" t="s">
+      <c r="B10" s="39" t="s">
         <v>106</v>
       </c>
-      <c r="C10" s="35" t="s">
+      <c r="C10" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="35" t="s">
+      <c r="D10" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="35"/>
-      <c r="F10" s="37">
+      <c r="E10" s="30"/>
+      <c r="F10" s="32">
         <v>8</v>
       </c>
     </row>
@@ -1721,17 +1727,17 @@
       <c r="A11" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="34" t="s">
+      <c r="B11" s="37" t="s">
         <v>109</v>
       </c>
-      <c r="C11" s="35" t="s">
+      <c r="C11" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="35" t="s">
+      <c r="D11" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="E11" s="35"/>
-      <c r="F11" s="37">
+      <c r="E11" s="30"/>
+      <c r="F11" s="32">
         <v>2</v>
       </c>
     </row>
@@ -1769,17 +1775,17 @@
       <c r="A15" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="B15" s="34" t="s">
+      <c r="B15" s="37" t="s">
         <v>110</v>
       </c>
-      <c r="C15" s="35" t="s">
+      <c r="C15" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="D15" s="35" t="s">
+      <c r="D15" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="E15" s="35"/>
-      <c r="F15" s="37">
+      <c r="E15" s="30"/>
+      <c r="F15" s="32">
         <v>4</v>
       </c>
     </row>
@@ -1790,14 +1796,14 @@
       <c r="B16" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="C16" s="35" t="s">
+      <c r="C16" s="30" t="s">
         <v>47</v>
       </c>
-      <c r="D16" s="35" t="s">
+      <c r="D16" s="30" t="s">
         <v>48</v>
       </c>
-      <c r="E16" s="35"/>
-      <c r="F16" s="37">
+      <c r="E16" s="30"/>
+      <c r="F16" s="32">
         <v>2</v>
       </c>
     </row>
@@ -1805,17 +1811,17 @@
       <c r="A17" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="B17" s="40" t="s">
+      <c r="B17" s="39" t="s">
         <v>106</v>
       </c>
-      <c r="C17" s="35" t="s">
+      <c r="C17" s="30" t="s">
         <v>52</v>
       </c>
-      <c r="D17" s="35" t="s">
+      <c r="D17" s="30" t="s">
         <v>53</v>
       </c>
-      <c r="E17" s="35"/>
-      <c r="F17" s="37">
+      <c r="E17" s="30"/>
+      <c r="F17" s="32">
         <v>5</v>
       </c>
       <c r="G17" s="12"/>
@@ -1828,13 +1834,13 @@
       <c r="A18" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="B18" s="40" t="s">
+      <c r="B18" s="39" t="s">
         <v>106</v>
       </c>
-      <c r="C18" s="35"/>
-      <c r="D18" s="35"/>
-      <c r="E18" s="35"/>
-      <c r="F18" s="37">
+      <c r="C18" s="30"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="32">
         <v>4</v>
       </c>
       <c r="G18" s="12"/>
@@ -1847,13 +1853,13 @@
       <c r="A19" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="B19" s="34" t="s">
+      <c r="B19" s="37" t="s">
         <v>112</v>
       </c>
-      <c r="C19" s="35"/>
-      <c r="D19" s="35"/>
-      <c r="E19" s="35"/>
-      <c r="F19" s="37">
+      <c r="C19" s="30"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="30"/>
+      <c r="F19" s="32">
         <v>3</v>
       </c>
       <c r="G19" s="12"/>
@@ -1866,13 +1872,13 @@
       <c r="A20" s="25" t="s">
         <v>57</v>
       </c>
-      <c r="B20" s="40" t="s">
+      <c r="B20" s="39" t="s">
         <v>106</v>
       </c>
-      <c r="C20" s="35"/>
-      <c r="D20" s="35"/>
-      <c r="E20" s="35"/>
-      <c r="F20" s="37">
+      <c r="C20" s="30"/>
+      <c r="D20" s="30"/>
+      <c r="E20" s="30"/>
+      <c r="F20" s="32">
         <v>3</v>
       </c>
       <c r="G20" s="12"/>
@@ -1885,13 +1891,13 @@
       <c r="A21" s="25" t="s">
         <v>58</v>
       </c>
-      <c r="B21" s="40" t="s">
+      <c r="B21" s="39" t="s">
         <v>106</v>
       </c>
-      <c r="C21" s="35"/>
-      <c r="D21" s="35"/>
-      <c r="E21" s="35"/>
-      <c r="F21" s="37">
+      <c r="C21" s="30"/>
+      <c r="D21" s="30"/>
+      <c r="E21" s="30"/>
+      <c r="F21" s="32">
         <v>4</v>
       </c>
       <c r="G21" s="12"/>
@@ -1904,13 +1910,13 @@
       <c r="A22" s="25" t="s">
         <v>59</v>
       </c>
-      <c r="B22" s="40" t="s">
+      <c r="B22" s="39" t="s">
         <v>106</v>
       </c>
-      <c r="C22" s="35"/>
-      <c r="D22" s="35"/>
-      <c r="E22" s="35"/>
-      <c r="F22" s="37">
+      <c r="C22" s="30"/>
+      <c r="D22" s="30"/>
+      <c r="E22" s="30"/>
+      <c r="F22" s="32">
         <v>1</v>
       </c>
       <c r="G22" s="12"/>
@@ -1926,10 +1932,10 @@
       <c r="B23" s="38" t="s">
         <v>113</v>
       </c>
-      <c r="C23" s="35"/>
-      <c r="D23" s="35"/>
-      <c r="E23" s="35"/>
-      <c r="F23" s="37">
+      <c r="C23" s="30"/>
+      <c r="D23" s="30"/>
+      <c r="E23" s="30"/>
+      <c r="F23" s="32">
         <v>5</v>
       </c>
       <c r="G23" s="12"/>
@@ -1942,13 +1948,13 @@
       <c r="A24" s="26" t="s">
         <v>61</v>
       </c>
-      <c r="B24" s="34" t="s">
+      <c r="B24" s="37" t="s">
         <v>114</v>
       </c>
-      <c r="C24" s="35"/>
-      <c r="D24" s="35"/>
-      <c r="E24" s="35"/>
-      <c r="F24" s="37">
+      <c r="C24" s="30"/>
+      <c r="D24" s="30"/>
+      <c r="E24" s="30"/>
+      <c r="F24" s="32">
         <v>9</v>
       </c>
     </row>
@@ -2302,11 +2308,11 @@
       <c r="A2" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="25" t="s">
@@ -2384,11 +2390,11 @@
       <c r="A8" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="B8" s="41"/>
-      <c r="C8" s="42"/>
-      <c r="D8" s="42"/>
-      <c r="E8" s="42"/>
-      <c r="F8" s="42"/>
+      <c r="B8" s="34"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="35"/>
+      <c r="E8" s="35"/>
+      <c r="F8" s="35"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" s="25" t="s">
@@ -2467,7 +2473,7 @@
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A13" s="43"/>
+      <c r="A13" s="36"/>
       <c r="B13" s="16"/>
       <c r="C13" s="9"/>
       <c r="D13" s="9"/>
@@ -2478,11 +2484,11 @@
       <c r="A14" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="B14" s="41"/>
-      <c r="C14" s="42"/>
-      <c r="D14" s="42"/>
-      <c r="E14" s="42"/>
-      <c r="F14" s="42"/>
+      <c r="B14" s="34"/>
+      <c r="C14" s="35"/>
+      <c r="D14" s="35"/>
+      <c r="E14" s="35"/>
+      <c r="F14" s="35"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A15" s="25" t="s">
@@ -2549,7 +2555,7 @@
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" s="43"/>
+      <c r="A19" s="36"/>
       <c r="B19" s="16"/>
       <c r="C19" s="9"/>
       <c r="D19" s="9"/>
@@ -2560,11 +2566,11 @@
       <c r="A20" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="B20" s="41"/>
-      <c r="C20" s="42"/>
-      <c r="D20" s="42"/>
-      <c r="E20" s="42"/>
-      <c r="F20" s="42"/>
+      <c r="B20" s="34"/>
+      <c r="C20" s="35"/>
+      <c r="D20" s="35"/>
+      <c r="E20" s="35"/>
+      <c r="F20" s="35"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="25" t="s">
@@ -2631,7 +2637,7 @@
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A25" s="43"/>
+      <c r="A25" s="36"/>
       <c r="B25" s="16"/>
       <c r="C25" s="9"/>
       <c r="D25" s="9"/>
@@ -2642,11 +2648,11 @@
       <c r="A26" s="14" t="s">
         <v>124</v>
       </c>
-      <c r="B26" s="41"/>
-      <c r="C26" s="42"/>
-      <c r="D26" s="42"/>
-      <c r="E26" s="42"/>
-      <c r="F26" s="42"/>
+      <c r="B26" s="34"/>
+      <c r="C26" s="35"/>
+      <c r="D26" s="35"/>
+      <c r="E26" s="35"/>
+      <c r="F26" s="35"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" s="25" t="s">
@@ -2713,7 +2719,7 @@
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A31" s="43"/>
+      <c r="A31" s="36"/>
       <c r="B31" s="16"/>
       <c r="C31" s="9"/>
       <c r="D31" s="9"/>
@@ -2724,11 +2730,11 @@
       <c r="A32" s="14" t="s">
         <v>125</v>
       </c>
-      <c r="B32" s="41"/>
-      <c r="C32" s="42"/>
-      <c r="D32" s="42"/>
-      <c r="E32" s="42"/>
-      <c r="F32" s="42"/>
+      <c r="B32" s="34"/>
+      <c r="C32" s="35"/>
+      <c r="D32" s="35"/>
+      <c r="E32" s="35"/>
+      <c r="F32" s="35"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" s="25" t="s">
@@ -2795,7 +2801,7 @@
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A37" s="43"/>
+      <c r="A37" s="36"/>
       <c r="B37" s="16"/>
       <c r="C37" s="9"/>
       <c r="D37" s="9"/>
@@ -2806,11 +2812,11 @@
       <c r="A38" s="14" t="s">
         <v>126</v>
       </c>
-      <c r="B38" s="41"/>
-      <c r="C38" s="42"/>
-      <c r="D38" s="42"/>
-      <c r="E38" s="42"/>
-      <c r="F38" s="42"/>
+      <c r="B38" s="34"/>
+      <c r="C38" s="35"/>
+      <c r="D38" s="35"/>
+      <c r="E38" s="35"/>
+      <c r="F38" s="35"/>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" s="25" t="s">
@@ -2877,7 +2883,7 @@
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A43" s="43"/>
+      <c r="A43" s="36"/>
       <c r="B43" s="16"/>
       <c r="C43" s="9"/>
       <c r="D43" s="9"/>
@@ -2888,11 +2894,11 @@
       <c r="A44" s="14" t="s">
         <v>124</v>
       </c>
-      <c r="B44" s="41"/>
-      <c r="C44" s="42"/>
-      <c r="D44" s="42"/>
-      <c r="E44" s="42"/>
-      <c r="F44" s="42"/>
+      <c r="B44" s="34"/>
+      <c r="C44" s="35"/>
+      <c r="D44" s="35"/>
+      <c r="E44" s="35"/>
+      <c r="F44" s="35"/>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" s="25" t="s">
@@ -2966,9 +2972,362 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9871143-4846-498A-9587-6847C2BB1359}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="81.6328125" customWidth="1"/>
+    <col min="2" max="2" width="21.6328125" customWidth="1"/>
+    <col min="3" max="3" width="25.1796875" customWidth="1"/>
+    <col min="4" max="4" width="26.90625" customWidth="1"/>
+    <col min="5" max="5" width="34.453125" customWidth="1"/>
+    <col min="6" max="6" width="13.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="B2" s="30" t="s">
+        <v>117</v>
+      </c>
+      <c r="C2" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="31" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="32">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" s="22" t="s">
+        <v>134</v>
+      </c>
+      <c r="B3" s="30" t="s">
+        <v>118</v>
+      </c>
+      <c r="C3" s="30" t="s">
+        <v>66</v>
+      </c>
+      <c r="D3" s="30" t="s">
+        <v>67</v>
+      </c>
+      <c r="E3" s="30" t="s">
+        <v>84</v>
+      </c>
+      <c r="F3" s="32">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" s="22" t="s">
+        <v>135</v>
+      </c>
+      <c r="B4" s="30" t="s">
+        <v>85</v>
+      </c>
+      <c r="C4" s="30" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="30" t="s">
+        <v>86</v>
+      </c>
+      <c r="F4" s="32">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" s="22" t="s">
+        <v>136</v>
+      </c>
+      <c r="B5" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="C5" s="30" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" s="32">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" s="22" t="s">
+        <v>137</v>
+      </c>
+      <c r="B6" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="30" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" s="32">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" s="22" t="s">
+        <v>138</v>
+      </c>
+      <c r="B7" s="30" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="30" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="30" t="s">
+        <v>29</v>
+      </c>
+      <c r="E7" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7" s="32">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" s="22" t="s">
+        <v>139</v>
+      </c>
+      <c r="B8" s="30" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" s="30" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" s="32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" s="22" t="s">
+        <v>140</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F9" s="10">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" s="22" t="s">
+        <v>75</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="F10" s="10">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" s="22" t="s">
+        <v>76</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" s="22" t="s">
+        <v>77</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="F12" s="10">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F13" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="F14" s="10">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" s="22" t="s">
+        <v>80</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="F15" s="10">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" s="22" t="s">
+        <v>81</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="F16" s="10">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A17" s="3"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="5"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A18" s="6"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>